<commit_message>
removed issue column from excel/csv site list export
</commit_message>
<xml_diff>
--- a/api/templates/export/sites/en.xlsx
+++ b/api/templates/export/sites/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26529"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\export\sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97AD6AD8-D96D-49EA-BF68-D11AA667EA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239DB878-2BA2-4FA1-BCEE-CF49AED3444E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sites" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>&lt;name&gt;</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Number of Devices</t>
   </si>
   <si>
-    <t>Issues</t>
-  </si>
-  <si>
     <t>&lt;totalDevices&gt;</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
   </si>
   <si>
     <t>Site Name</t>
-  </si>
-  <si>
-    <t>&lt;siteIssues&gt;</t>
   </si>
   <si>
     <t>&lt;Table&gt;</t>
@@ -143,16 +137,29 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color auto="1"/>
       </left>
       <right style="thin">
         <color auto="1"/>
       </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="medium">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -167,22 +174,7 @@
       <top style="medium">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -191,13 +183,13 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -248,7 +240,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -256,26 +248,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -686,219 +681,210 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J29"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.19921875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="37.25" style="2" customWidth="1"/>
     <col min="2" max="2" width="21.5" style="1" customWidth="1"/>
-    <col min="3" max="4" width="25.59765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.09765625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="32" style="1" customWidth="1"/>
+    <col min="3" max="4" width="25.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.75" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="4" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="3" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+    </row>
+    <row r="6" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-    </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-    </row>
-    <row r="21" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-    </row>
-    <row r="22" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-    </row>
-    <row r="23" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-    </row>
-    <row r="24" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-    </row>
-    <row r="25" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-    </row>
-    <row r="26" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-    </row>
-    <row r="27" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-    </row>
-    <row r="28" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-    </row>
-    <row r="29" spans="7:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>